<commit_message>
Verifica settimanale: deduplica cross-file (59 duplicati marcati nei nuovi file, 10 in file preesistenti mai deduplicati)
Deduplica globale su tutti i 180 file xlsx in /output basata su ragione_sociale
normalizzata e dominio del sito web (incl. path per distinguere filiali/dealer
sulla stessa piattaforma). Le occorrenze piu recenti vengono annotate nel campo
note con "[DUPLICATO — vedi anche: <file canonico>]" senza modificare le righe
canoniche ne cancellare alcuna riga.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014CgvovxTrdARiZ1ujqwH5a
</commit_message>
<xml_diff>
--- a/output/2026-09-03_13_Italia_Campania_Metalworking_Lavorazioni_Metalliche.xlsx
+++ b/output/2026-09-03_13_Italia_Campania_Metalworking_Lavorazioni_Metalliche.xlsx
@@ -1077,7 +1077,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Impianti di aspirazione, due sedi in Campania. Sito web non reperito; tipologia impianti (industriale vs civile) non verificabile online, da confermare umanamente.</t>
+          <t>Impianti di aspirazione, due sedi in Campania. Sito web non reperito; tipologia impianti (industriale vs civile) non verificabile online, da confermare umanamente. [DUPLICATO — vedi anche: 2026-09-03_01_Italia_Campania_Depolverazione_Trattamento_aria.xlsx]</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Condizionamento e aspirazione; target civile o industriale non specificato nella fonte, sito web non reperito. Da confermare umanamente prima dell'uso commerciale.</t>
+          <t>Condizionamento e aspirazione; target civile o industriale non specificato nella fonte, sito web non reperito. Da confermare umanamente prima dell'uso commerciale. [DUPLICATO — vedi anche: 2026-09-03_02_Italia_Campania_Impiantistica_aspirazione_industriale.xlsx]</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">

</xml_diff>